<commit_message>
feat: refresh waybill data to 612 records
🌐 - Generated by Copilot
</commit_message>
<xml_diff>
--- a/运单段码对照表.xlsx
+++ b/运单段码对照表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13605"/>
+    <workbookView windowWidth="28800" windowHeight="11805"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="640">
   <si>
     <t>运单号</t>
   </si>
@@ -1929,6 +1929,24 @@
   </si>
   <si>
     <t>JDM000002716722</t>
+  </si>
+  <si>
+    <t>JDM000004648942</t>
+  </si>
+  <si>
+    <t>JDM000004302515</t>
+  </si>
+  <si>
+    <t>JDM000003736095</t>
+  </si>
+  <si>
+    <t>JDM000002861416</t>
+  </si>
+  <si>
+    <t>JDM000001931730</t>
+  </si>
+  <si>
+    <t>JDM000003187445</t>
   </si>
 </sst>
 </file>
@@ -2695,7 +2713,14 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2889,25 +2914,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="totalRow" dxfId="5"/>
+      <tableStyleElement type="firstColumn" dxfId="4"/>
+      <tableStyleElement type="lastColumn" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="17"/>
+      <tableStyleElement type="totalRow" dxfId="16"/>
+      <tableStyleElement type="firstRowStripe" dxfId="15"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="14"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="13"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="11"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="10"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="9"/>
+      <tableStyleElement type="pageFieldValues" dxfId="8"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3168,7 +3193,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B607"/>
+  <dimension ref="A1:B619"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="26.125" customWidth="1"/>
@@ -8031,7 +8056,79 @@
         <v>8</v>
       </c>
     </row>
+    <row r="608" spans="1:2">
+      <c r="A608" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="B608" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="609" spans="1:2">
+      <c r="A609" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="B609" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="610" spans="1:2">
+      <c r="A610" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="B610" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="611" spans="1:2">
+      <c r="A611" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="B611" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="612" spans="1:2">
+      <c r="A612" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="B612" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="613" spans="1:2">
+      <c r="A613" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="B613" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="614" spans="1:2">
+      <c r="A614" s="3"/>
+      <c r="B614" s="4"/>
+    </row>
+    <row r="615" spans="1:2">
+      <c r="A615" s="3"/>
+      <c r="B615" s="4"/>
+    </row>
+    <row r="616" spans="1:2">
+      <c r="A616" s="3"/>
+      <c r="B616" s="4"/>
+    </row>
+    <row r="617" spans="1:2">
+      <c r="A617" s="3"/>
+    </row>
+    <row r="618" spans="1:2">
+      <c r="A618" s="3"/>
+    </row>
+    <row r="619" spans="1:2">
+      <c r="A619" s="3"/>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A$1:A$1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
feat: refresh waybill segment data
🌐 - Generated by Copilot
</commit_message>
<xml_diff>
--- a/运单段码对照表.xlsx
+++ b/运单段码对照表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11805"/>
+    <workbookView windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3193,7 +3193,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B619"/>
+  <dimension ref="A1:B613"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="26.125" customWidth="1"/>
@@ -8061,7 +8061,7 @@
         <v>634</v>
       </c>
       <c r="B608" s="4" t="s">
-        <v>19</v>
+        <v>71</v>
       </c>
     </row>
     <row r="609" spans="1:2">
@@ -8085,7 +8085,7 @@
         <v>637</v>
       </c>
       <c r="B611" s="4" t="s">
-        <v>209</v>
+        <v>71</v>
       </c>
     </row>
     <row r="612" spans="1:2">
@@ -8103,27 +8103,6 @@
       <c r="B613" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="614" spans="1:2">
-      <c r="A614" s="3"/>
-      <c r="B614" s="4"/>
-    </row>
-    <row r="615" spans="1:2">
-      <c r="A615" s="3"/>
-      <c r="B615" s="4"/>
-    </row>
-    <row r="616" spans="1:2">
-      <c r="A616" s="3"/>
-      <c r="B616" s="4"/>
-    </row>
-    <row r="617" spans="1:2">
-      <c r="A617" s="3"/>
-    </row>
-    <row r="618" spans="1:2">
-      <c r="A618" s="3"/>
-    </row>
-    <row r="619" spans="1:2">
-      <c r="A619" s="3"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A$1:A$1048576">

</xml_diff>